<commit_message>
PX-14: add release gate report and update docs/spreadsheet/scripts
</commit_message>
<xml_diff>
--- a/output/spreadsheet/px11-advanced-report.xlsx
+++ b/output/spreadsheet/px11-advanced-report.xlsx
@@ -429,7 +429,7 @@
         <v>تاريخ التوليد</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-03-11T10:30:40.492Z</v>
+        <v>2026-03-11T20:47:22.890Z</v>
       </c>
       <c r="C2" t="str">
         <v/>
@@ -765,7 +765,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>AYA-2026-39850</v>
+        <v>AYA-2026-42423</v>
       </c>
       <c r="B2" t="str">
         <v>2026-03-11</v>
@@ -839,7 +839,7 @@
         <v>12</v>
       </c>
       <c r="F2" t="str">
-        <v>مصروف AYA-2026-39950 — PX11 current expense</v>
+        <v>مصروف AYA-2026-42475 — PX11 current expense</v>
       </c>
     </row>
     <row r="3">
@@ -859,7 +859,7 @@
         <v>200</v>
       </c>
       <c r="F3" t="str">
-        <v>فاتورة بيع AYA-2026-39850</v>
+        <v>فاتورة بيع AYA-2026-42423</v>
       </c>
     </row>
   </sheetData>
@@ -911,7 +911,7 @@
         <v>1</v>
       </c>
       <c r="E2" t="str">
-        <v>2026-03-11T10:30:40.06961+00:00</v>
+        <v>2026-03-11T20:47:22.403231+00:00</v>
       </c>
     </row>
     <row r="3">
@@ -928,7 +928,7 @@
         <v>1</v>
       </c>
       <c r="E3" t="str">
-        <v>2026-03-11T10:30:39.979653+00:00</v>
+        <v>2026-03-11T20:47:22.351365+00:00</v>
       </c>
     </row>
   </sheetData>

</xml_diff>